<commit_message>
Day 2 Deliverables comitted
</commit_message>
<xml_diff>
--- a/Anumoy_Pathak_RedBus/Bus_Seat_Booking_Test_Scenarios_Updated.xlsx
+++ b/Anumoy_Pathak_RedBus/Bus_Seat_Booking_Test_Scenarios_Updated.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d6a5426fd29e00d/Desktop/Sprint/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d6a5426fd29e00d/Desktop/Anumoy_Pathak_RedBus/Anumoy_Pathak_RedBus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD22E0BC-8CC8-4D9B-B858-6C0424C027E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{BD22E0BC-8CC8-4D9B-B858-6C0424C027E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{503C4BB7-5E3C-4EF6-81BE-79F59BF80C02}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -71,12 +71,6 @@
     <t>Verify seat layout details including deck view and seat type display</t>
   </si>
   <si>
-    <t>1. Validate both lower and upper deck are displayed for sleeper buses
-2. Validate only a single deck is shown for non-sleeper buses
-3. Validate window and aisle seat labels are correctly shown for each seat
-4. Validate seat type icons/labels are visible and distinct</t>
-  </si>
-  <si>
     <t>TS_BusSeat_03</t>
   </si>
   <si>
@@ -195,11 +189,16 @@
     <t>Verify invalid age error handling and auto-fill from saved profile</t>
   </si>
   <si>
+    <t>1. Validate both lower and upper deck are displayed for sleeper buses
+2. Validate only a single deck is shown for non-sleeper buses
+3. Validate seat type icons/labels are visible and distinct</t>
+  </si>
+  <si>
     <t>1. Validate entering age as 0 or a negative number shows an appropriate error
 2. Validate entering age above 120 shows an appropriate error
 3. Validate entering text in the age field shows an error message
-4. Validate auto-fill populates name, age and gender from the saved profile
-5. Validate auto-filled details can be manually edited and auto-fill is not triggered if no profile is saved</t>
+4. Fill the contact details
+5. Proceed to the payments page and validate the payment functionalities</t>
   </si>
 </sst>
 </file>
@@ -219,10 +218,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -307,6 +308,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -659,21 +664,21 @@
         <v>9</v>
       </c>
       <c r="E3" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
@@ -682,18 +687,18 @@
         <v>4</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>9</v>
@@ -702,18 +707,18 @@
         <v>5</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>9</v>
@@ -722,18 +727,18 @@
         <v>5</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>9</v>
@@ -742,18 +747,18 @@
         <v>4</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
@@ -762,18 +767,18 @@
         <v>4</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>9</v>
@@ -782,18 +787,18 @@
         <v>3</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>9</v>
@@ -802,18 +807,18 @@
         <v>7</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>9</v>

</xml_diff>